<commit_message>
Part 4 ecomatik analysis
</commit_message>
<xml_diff>
--- a/Ecomatik/raw_data_DSCMET422/DSCMET422_metadata.xlsx
+++ b/Ecomatik/raw_data_DSCMET422/DSCMET422_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabby\Desktop\GJ_OSU_Thesis\GJ_OSU_Thesis\Ecomatik\raw_data_DSCMET422\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0091EB8E-945E-48CA-AEC7-871452B94BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8934BF5F-8BC8-469A-B3DE-64D6C6981164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{22CF2F88-BCF7-4A13-BA2E-9C967ACC2069}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{22CF2F88-BCF7-4A13-BA2E-9C967ACC2069}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>